<commit_message>
Final improvements: enhanced regex patterns and added usage examples
Co-authored-by: Tanziwei <18663157+Tanziwei@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/function_documentation.xlsx
+++ b/function_documentation.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -702,6 +702,58 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EDGE_CASE_001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MinimalFunction</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>void MinimalFunction(void);</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EDGE_CASE_002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ComplexReturnFunction</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>const volatile uint32* ComplexReturnFunction(const uint8* data);</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>参数名：data
+输入/输出：输入
+值域范围：Valid pointer
+初始值：NULL
+说明：Data to process</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>类型：const volatile uint32*
+值域范围：Valid pointer or NULL
+说明：Pointer to processed data result</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>